<commit_message>
Update Cost declines by tech.xlsx
</commit_message>
<xml_diff>
--- a/data/Cost declines by tech.xlsx
+++ b/data/Cost declines by tech.xlsx
@@ -8,24 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9a072a59b81ab8f9/Documents/Work/Clients ^0 prospects/EpochAI/inference-cost/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1390" documentId="8_{237EF59B-240D-4B45-BBDB-12EDD86E70D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A1BBF066-C0FE-4E31-A20B-81B5F83AE3B0}"/>
+  <xr:revisionPtr revIDLastSave="1440" documentId="8_{237EF59B-240D-4B45-BBDB-12EDD86E70D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D9B9F86-9EF2-40D1-AB39-4F0EB1DD6042}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="14592" activeTab="1" xr2:uid="{55FDA7DF-2265-4D1B-B569-857BE3FE3144}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="14592" xr2:uid="{55FDA7DF-2265-4D1B-B569-857BE3FE3144}"/>
   </bookViews>
   <sheets>
-    <sheet name="Chart1" sheetId="10" r:id="rId1"/>
-    <sheet name="Table" sheetId="4" r:id="rId2"/>
-    <sheet name="Figure data" sheetId="9" r:id="rId3"/>
-    <sheet name="Electricity" sheetId="8" r:id="rId4"/>
-    <sheet name="Illumination" sheetId="6" r:id="rId5"/>
-    <sheet name="Lithium batteries" sheetId="5" r:id="rId6"/>
-    <sheet name="Compute" sheetId="7" r:id="rId7"/>
-    <sheet name="DNA sequencing" sheetId="1" r:id="rId8"/>
-    <sheet name="CPI" sheetId="3" r:id="rId9"/>
-    <sheet name="Sources" sheetId="2" r:id="rId10"/>
+    <sheet name="Figure" sheetId="4" r:id="rId1"/>
+    <sheet name="Figure data" sheetId="9" r:id="rId2"/>
+    <sheet name="Electricity" sheetId="8" r:id="rId3"/>
+    <sheet name="Illumination" sheetId="6" r:id="rId4"/>
+    <sheet name="Lithium batteries" sheetId="5" r:id="rId5"/>
+    <sheet name="Compute" sheetId="7" r:id="rId6"/>
+    <sheet name="DNA sequencing" sheetId="1" r:id="rId7"/>
+    <sheet name="CPI" sheetId="3" r:id="rId8"/>
+    <sheet name="Sources" sheetId="2" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Electricity!$A$6:$B$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Electricity!$A$6:$B$140</definedName>
     <definedName name="fn">'DNA sequencing'!$J$20</definedName>
     <definedName name="Year_span">'DNA sequencing'!$I$1</definedName>
   </definedNames>
@@ -75,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2057" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2059" uniqueCount="238">
   <si>
     <t>World</t>
   </si>
@@ -2308,6 +2307,12 @@
   <si>
     <t>LLM t</t>
   </si>
+  <si>
+    <t>Relative to AI</t>
+  </si>
+  <si>
+    <t>x/year</t>
+  </si>
 </sst>
 </file>
 
@@ -2521,7 +2526,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2680,6 +2685,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2856,1878 +2873,9 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="9.4016404945968773E-2"/>
+          <c:x val="0.15474459887663092"/>
           <c:y val="6.0274498584973017E-2"/>
-          <c:w val="0.86806932836467099"/>
-          <c:h val="0.83039405742350791"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="7"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:v>AI</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="12700" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>'Figure data'!$M$3:$M$4</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-                <c:pt idx="0">
-                  <c:v>1.6163586584530094</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>4.7829586584530261</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>'Figure data'!$N$3:$N$4</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-                <c:pt idx="0">
-                  <c:v>1.6493911422653169E-2</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>5.307518695827581E-6</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-28D7-4073-BEF6-C7AC152E9096}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="3"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>Compute</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="12700" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent4"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>'Figure data'!$G$2:$G$56</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="55"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>6</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>8</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>12</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>13</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>15</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>18</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>19</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>21</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>22</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>23</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>24</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>26</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>27</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>29</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>30</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>31</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>32</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>33</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>35</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>36</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>37</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>38</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>40</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>42</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>43</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>44</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>45</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>46</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>47</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>48</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>51</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>52</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>53</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>54</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>55</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>56</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>57</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>58</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>59</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>60</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>61</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>'Figure data'!$H$2:$H$56</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="55"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.35115476038867788</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>7.8033172753900662E-2</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>7.8033172753900662E-2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>7.8033172753900662E-2</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>4.6382056926548551E-2</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>4.6382056926548551E-2</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>4.6382056926548551E-2</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>5.7840715825846489E-3</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>5.7840715825846489E-3</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>5.7840715825846489E-3</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>5.7840715825846489E-3</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>1.1894462989462484E-3</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>1.1894462989462484E-3</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>3.9869035438097036E-4</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>3.9869035438097036E-4</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>3.9869035438097036E-4</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>1.4230696120937078E-4</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>1.3078890527653685E-4</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>1.3078890527653685E-4</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>1.3078890527653685E-4</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>4.4641876916147174E-5</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>4.4641876916147174E-5</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>4.4641876916147174E-5</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>4.4641876916147174E-5</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>2.3236862295869747E-5</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>2.3236862295869747E-5</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>2.3236862295869747E-5</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>2.3236862295869747E-5</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>2.3236862295869747E-5</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>2.3236862295869747E-5</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>3.1618192756799012E-6</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>7.2772030948188204E-7</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>7.2772030948188204E-7</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>7.2772030948188204E-7</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>1.2546901887618653E-7</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>1.2546901887618653E-7</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>1.2546901887618653E-7</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>1.2546901887618653E-7</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>2.5093803775237309E-8</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>2.5093803775237309E-8</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>4.7678227172950891E-9</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>4.7678227172950891E-9</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>1.5056282265142386E-9</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>1.5056282265142386E-9</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>5.0187607550474615E-10</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>2.5093803775237307E-10</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>2.5093803775237307E-10</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>2.5093803775237307E-10</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>2.5093803775237307E-10</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>5.9723252985064788E-11</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>3.7389767625103589E-11</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>3.7389767625103589E-11</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>1.026336574407206E-11</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-28D7-4073-BEF6-C7AC152E9096}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:v>Lithium batteries</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="12700" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>'Figure data'!$D$2:$D$35</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="34"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>6</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>8</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>12</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>13</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>15</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>16</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>17</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>18</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>19</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>21</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>22</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>23</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>24</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>26</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>27</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>28</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>29</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>30</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>31</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>32</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>33</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>'Figure data'!$E$2:$E$35</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="34"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.80216650398524247</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.63861393255108734</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.72902084964219138</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.68422648511492123</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.57629766031901486</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.49350477675367499</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0.39704364603272668</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0.30073870033647371</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0.29213463724575828</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0.20390688397575304</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0.14609075994844864</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0.11295786315868334</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0.10107282119990488</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>8.7135380983971084E-2</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>7.462309193147186E-2</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>7.1207342270497048E-2</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>7.4662293992658169E-2</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>6.6510416135101946E-2</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>5.9794450301458274E-2</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>5.6958182368952774E-2</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>5.8597070865765571E-2</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>5.3298723267497128E-2</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>4.7150820337820011E-2</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>3.6040658050884723E-2</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>2.8120904689676589E-2</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>2.0303510335789657E-2</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>1.7046262688336773E-2</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>1.4331889648792702E-2</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>1.3354715354556837E-2</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>1.2920415668229785E-2</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>1.4331889648792702E-2</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>1.2051816295575682E-2</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>8.468843883377505E-3</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-28D7-4073-BEF6-C7AC152E9096}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="3"/>
-          <c:tx>
-            <c:v>DNA sequencing</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="12700" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>'Figure data'!$J$2:$J$79</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="78"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.49828884325802392</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.99931553730334599</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1.4976043805613699</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>2.0835044490077053</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>2.3353867214236743</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2.5817932922657292</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>2.8336755646816982</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>3.0855578370978947</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>3.3374401095140911</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>3.5811088295688478</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>3.8329911019850442</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>4.0848733744012407</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>4.3367556468174371</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>4.5804243668721938</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>4.8323066392881628</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>5.0841889117043593</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>5.3360711841205557</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>5.5797399041753124</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>5.8316221765915088</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>6.0835044490077053</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>6.3353867214236743</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>6.5817932922657292</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>6.8336755646816982</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>7.0855578370978947</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>7.3374401095140911</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>7.5811088295688478</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>7.8329911019850442</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>8.0848733744012407</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>8.3367556468174371</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>8.5804243668721938</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>8.8323066392881628</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>9.0841889117043593</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>9.3360711841205557</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>9.5797399041753124</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>9.8316221765915088</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>10.080766598220407</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>10.335386721423674</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>10.581793292265729</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>10.833675564681698</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>11.085557837097895</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>11.337440109514091</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>11.581108829568848</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>11.832991101985044</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>12.084873374401241</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>12.336755646817437</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>12.580424366872194</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>12.832306639288163</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>13.084188911704359</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>13.336071184120556</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>13.579739904175312</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>13.831622176591509</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>14.083504449007705</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>14.666666666666742</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>14.918548939082939</c:v>
-                </c:pt>
-                <c:pt idx="55">
-                  <c:v>15.167693360711837</c:v>
-                </c:pt>
-                <c:pt idx="56">
-                  <c:v>15.414099931553892</c:v>
-                </c:pt>
-                <c:pt idx="57">
-                  <c:v>15.665982203969861</c:v>
-                </c:pt>
-                <c:pt idx="58">
-                  <c:v>15.917864476386058</c:v>
-                </c:pt>
-                <c:pt idx="59">
-                  <c:v>16.167008898015183</c:v>
-                </c:pt>
-                <c:pt idx="60">
-                  <c:v>16.413415468857011</c:v>
-                </c:pt>
-                <c:pt idx="61">
-                  <c:v>16.665297741273207</c:v>
-                </c:pt>
-                <c:pt idx="62">
-                  <c:v>16.917180013689403</c:v>
-                </c:pt>
-                <c:pt idx="63">
-                  <c:v>17.166324435318302</c:v>
-                </c:pt>
-                <c:pt idx="64">
-                  <c:v>17.412731006160357</c:v>
-                </c:pt>
-                <c:pt idx="65">
-                  <c:v>17.582477754962383</c:v>
-                </c:pt>
-                <c:pt idx="66">
-                  <c:v>17.83436002737858</c:v>
-                </c:pt>
-                <c:pt idx="67">
-                  <c:v>18.165639972621648</c:v>
-                </c:pt>
-                <c:pt idx="68">
-                  <c:v>18.412046543463475</c:v>
-                </c:pt>
-                <c:pt idx="69">
-                  <c:v>18.666666666666742</c:v>
-                </c:pt>
-                <c:pt idx="70">
-                  <c:v>18.918548939082939</c:v>
-                </c:pt>
-                <c:pt idx="71">
-                  <c:v>19.167693360711837</c:v>
-                </c:pt>
-                <c:pt idx="72">
-                  <c:v>19.414099931553892</c:v>
-                </c:pt>
-                <c:pt idx="73">
-                  <c:v>19.665982203969861</c:v>
-                </c:pt>
-                <c:pt idx="74">
-                  <c:v>19.917864476386058</c:v>
-                </c:pt>
-                <c:pt idx="75">
-                  <c:v>20.167008898015183</c:v>
-                </c:pt>
-                <c:pt idx="76">
-                  <c:v>20.413415468857011</c:v>
-                </c:pt>
-                <c:pt idx="77">
-                  <c:v>20.665297741273207</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>'Figure data'!$K$2:$K$79</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="78"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.72966450166975194</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.63222391132945199</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.54699705192006998</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.40468201668292464</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.2873892560087431</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.20250436288913715</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0.1964261179806801</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0.18010307127461045</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0.16990976065198432</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0.1556131540651009</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0.15382443136010684</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0.12988182068984197</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0.1176709291497095</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0.10865918549877641</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>0.10479033872157595</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>9.6672432806743716E-2</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>8.5889241079984052E-2</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>8.157688002031134E-2</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>8.0144379342313013E-2</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>6.320278748727777E-2</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>2.6855959871058328E-2</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>1.1720659796107069E-2</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>6.411408344161644E-3</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>2.9956434297798685E-3</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>2.0398733178367294E-3</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>1.3540116803166067E-3</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>9.3512050058278519E-4</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>6.0360355326899353E-4</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>4.0133189210794686E-4</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>2.7036791526076814E-4</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>2.662711554270181E-4</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>2.4698775629687983E-4</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>1.7612212416533382E-4</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>1.3859234684711133E-4</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>8.6550335982576426E-5</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>6.3548184017738271E-5</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>6.2594839264667776E-5</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>4.8103278850098872E-5</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>4.8527658871325301E-5</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>5.3356606328380226E-5</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>4.5390613351393476E-5</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>4.4621528929781469E-5</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>4.4322785484690122E-5</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>4.0583822454023445E-5</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>3.172342788152098E-5</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>3.8719458844008944E-5</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>3.8508215680075617E-5</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>4.5084089040370574E-5</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>3.1447903655264528E-5</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>3.3123140454630736E-5</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>1.0677107071392571E-5</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>9.7541058846892562E-6</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>9.1246967031509706E-6</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>1.1655187674886646E-5</c:v>
-                </c:pt>
-                <c:pt idx="55">
-                  <c:v>1.0417268640705677E-5</c:v>
-                </c:pt>
-                <c:pt idx="56">
-                  <c:v>7.761601513369908E-6</c:v>
-                </c:pt>
-                <c:pt idx="57">
-                  <c:v>1.0181197746957041E-5</c:v>
-                </c:pt>
-                <c:pt idx="58">
-                  <c:v>8.5785382607503547E-6</c:v>
-                </c:pt>
-                <c:pt idx="59">
-                  <c:v>1.3873546008372642E-5</c:v>
-                </c:pt>
-                <c:pt idx="60">
-                  <c:v>9.2049523124533013E-6</c:v>
-                </c:pt>
-                <c:pt idx="61">
-                  <c:v>1.0866685918468429E-5</c:v>
-                </c:pt>
-                <c:pt idx="62">
-                  <c:v>1.0847204116506927E-5</c:v>
-                </c:pt>
-                <c:pt idx="63">
-                  <c:v>1.0264509761350724E-5</c:v>
-                </c:pt>
-                <c:pt idx="64">
-                  <c:v>7.2814851439087127E-6</c:v>
-                </c:pt>
-                <c:pt idx="65">
-                  <c:v>4.4276553363266953E-6</c:v>
-                </c:pt>
-                <c:pt idx="66">
-                  <c:v>6.8601844627310086E-6</c:v>
-                </c:pt>
-                <c:pt idx="67">
-                  <c:v>5.0125444788007422E-6</c:v>
-                </c:pt>
-                <c:pt idx="68">
-                  <c:v>4.6566339492538819E-6</c:v>
-                </c:pt>
-                <c:pt idx="69">
-                  <c:v>5.0883900051850262E-6</c:v>
-                </c:pt>
-                <c:pt idx="70">
-                  <c:v>4.9373666442219515E-6</c:v>
-                </c:pt>
-                <c:pt idx="71">
-                  <c:v>3.6423861203251413E-6</c:v>
-                </c:pt>
-                <c:pt idx="72">
-                  <c:v>5.9866651559596355E-6</c:v>
-                </c:pt>
-                <c:pt idx="73">
-                  <c:v>3.1275476067508102E-6</c:v>
-                </c:pt>
-                <c:pt idx="74">
-                  <c:v>3.8263289384250511E-6</c:v>
-                </c:pt>
-                <c:pt idx="75">
-                  <c:v>3.6656030166835175E-6</c:v>
-                </c:pt>
-                <c:pt idx="76">
-                  <c:v>3.3999026951282636E-6</c:v>
-                </c:pt>
-                <c:pt idx="77">
-                  <c:v>3.3159531996810656E-6</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-28D7-4073-BEF6-C7AC152E9096}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="4"/>
-          <c:order val="4"/>
-          <c:tx>
-            <c:v>AI</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="12700" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>'Figure data'!$M$2:$M$3</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1.6163586584530094</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>'Figure data'!$N$2:$N$3</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1.6493911422653169E-2</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-28D7-4073-BEF6-C7AC152E9096}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="5"/>
-          <c:tx>
-            <c:v>Electricity</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="12700" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>'Figure data'!$A$2:$A$56</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="55"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>15</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>30</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>34</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>35</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>36</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>37</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>38</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>39</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>40</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>41</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>42</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>43</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>44</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>45</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>46</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>47</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>48</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>49</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>51</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>52</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>53</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>54</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>55</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>56</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>57</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>58</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>59</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>60</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>61</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>62</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>63</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>64</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>65</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>66</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>67</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>68</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>69</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>70</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>71</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>72</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>73</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>74</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>75</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>76</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>77</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>78</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>79</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>80</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>81</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>'Figure data'!$B$2:$B$56</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="55"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.98103137396321638</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.77924442228328306</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.46036688553442084</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.38533537553467684</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.24215681818181811</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.1810655844155844</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0.16300975860297892</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0.16155632183908042</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0.15981084529505579</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0.15257958532695373</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0.14882972237343495</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0.15673755980861243</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0.1687839416058394</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0.1750187412587412</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>0.16394993215739484</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>0.1507321831453218</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>0.13848122956180506</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>0.12279583333333331</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>0.12102359767891679</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>0.11861347285807716</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>0.11305558441558441</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>0.10458763141620282</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>9.3056999442275495E-2</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>8.5771939043615339E-2</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>8.2202169421487573E-2</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>7.8085555555555533E-2</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>6.8062843822843819E-2</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>5.7113982878108427E-2</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>5.1479969822708395E-2</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>5.1089763177998473E-2</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>4.9256582421727632E-2</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>4.4547342657342649E-2</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>4.3084665523156082E-2</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>4.2298808307797066E-2</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>4.1218181818181814E-2</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>4.0602985074626868E-2</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>3.9399732620320857E-2</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>3.7551083791653179E-2</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>3.6083737024221442E-2</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>3.541080912214932E-2</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>3.4394901719901713E-2</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>3.3774095469747648E-2</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>3.2892655027092113E-2</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>3.1923885918003561E-2</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>3.0714193548387093E-2</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>2.9441558441558432E-2</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>2.798765432098765E-2</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>2.6779477408818718E-2</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>2.5109926854754439E-2</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>2.3473024523160756E-2</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>2.2308809746954081E-2</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>2.2288350168350166E-2</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>2.2581252718573294E-2</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>2.209443079443079E-2</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-28D7-4073-BEF6-C7AC152E9096}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="1131568655"/>
-        <c:axId val="1321391791"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="1131568655"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1"/>
-                    </a:solidFill>
-                    <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                    <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US">
-                    <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-                    <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-                  </a:rPr>
-                  <a:t>Years since start of price decline</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
-        <c:numFmt formatCode="0" sourceLinked="0"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1"/>
-                </a:solidFill>
-                <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-                <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1321391791"/>
-        <c:crossesAt val="1.0000000000000006E-11"/>
-        <c:crossBetween val="midCat"/>
-        <c:majorUnit val="30"/>
-        <c:minorUnit val="10"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="1321391791"/>
-        <c:scaling>
-          <c:logBase val="10"/>
-          <c:orientation val="minMax"/>
-          <c:max val="1.05"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="none"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:noFill/>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1"/>
-                </a:solidFill>
-                <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1131568655"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln w="25400">
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:noFill/>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr sz="1100">
-          <a:solidFill>
-            <a:schemeClr val="tx1"/>
-          </a:solidFill>
-          <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-          <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-        </a:defRPr>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:userShapes r:id="rId3"/>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:autoTitleDeleted val="1"/>
-    <c:plotArea>
-      <c:layout>
-        <c:manualLayout>
-          <c:layoutTarget val="inner"/>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="9.4016404945968773E-2"/>
-          <c:y val="6.0274498584973017E-2"/>
-          <c:w val="0.86806932836467099"/>
+          <c:w val="0.80734109673495824"/>
           <c:h val="0.84656994233186922"/>
         </c:manualLayout>
       </c:layout>
@@ -6368,6 +4516,20 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
         <c:title>
           <c:tx>
             <c:rich>
@@ -6560,7 +4722,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -8415,7 +6577,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -9053,46 +7215,6 @@
 </file>
 
 <file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -10680,1471 +8802,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/chartsheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{B2ECE642-63CB-49BA-A3A9-08DA64A8BA4C}">
-  <sheetPr/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</chartsheet>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:absoluteAnchor>
-    <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8666825" cy="6292049"/>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0900A08B-AAD3-0CDF-DA80-ACFD86DA6F79}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr>
-          <a:graphicFrameLocks noGrp="1"/>
-        </xdr:cNvGraphicFramePr>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:absoluteAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
-    <cdr:from>
-      <cdr:x>0.67193</cdr:x>
-      <cdr:y>0.81426</cdr:y>
-    </cdr:from>
-    <cdr:to>
-      <cdr:x>0.8136</cdr:x>
-      <cdr:y>0.92661</cdr:y>
-    </cdr:to>
-    <cdr:sp macro="" textlink="">
-      <cdr:nvSpPr>
-        <cdr:cNvPr id="2" name="TextBox 1">
-          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2D886207-E4F1-F019-14A4-3966205D2678}"/>
-            </a:ext>
-          </a:extLst>
-        </cdr:cNvPr>
-        <cdr:cNvSpPr txBox="1"/>
-      </cdr:nvSpPr>
-      <cdr:spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="4500571" y="3196437"/>
-          <a:ext cx="948902" cy="441038"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </cdr:spPr>
-      <cdr:txBody>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-            <a:t>Compute</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:effectLst/>
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>,</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100">
-              <a:effectLst/>
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:effectLst/>
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>1940–2001</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" kern="1200">
-            <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </cdr:txBody>
-    </cdr:sp>
-  </cdr:relSizeAnchor>
-  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
-    <cdr:from>
-      <cdr:x>0.387</cdr:x>
-      <cdr:y>0.1999</cdr:y>
-    </cdr:from>
-    <cdr:to>
-      <cdr:x>0.52868</cdr:x>
-      <cdr:y>0.2709</cdr:y>
-    </cdr:to>
-    <cdr:sp macro="" textlink="">
-      <cdr:nvSpPr>
-        <cdr:cNvPr id="3" name="TextBox 1">
-          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A081233B-3C5D-69F2-6F98-E93F2A94B7BA}"/>
-            </a:ext>
-          </a:extLst>
-        </cdr:cNvPr>
-        <cdr:cNvSpPr txBox="1"/>
-      </cdr:nvSpPr>
-      <cdr:spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="2592123" y="784726"/>
-          <a:ext cx="948970" cy="278716"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </cdr:spPr>
-      <cdr:txBody>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="none" rtlCol="0"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:lvl1pPr marL="0" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl1pPr>
-          <a:lvl2pPr marL="457200" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl2pPr>
-          <a:lvl3pPr marL="914400" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl3pPr>
-          <a:lvl4pPr marL="1371600" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl4pPr>
-          <a:lvl5pPr marL="1828800" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl5pPr>
-          <a:lvl6pPr marL="2286000" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl6pPr>
-          <a:lvl7pPr marL="2743200" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl7pPr>
-          <a:lvl8pPr marL="3200400" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl8pPr>
-          <a:lvl9pPr marL="3657600" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl9pPr>
-        </a:lstStyle>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-            <a:t>Lithium</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-            <a:t>batteries</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:effectLst/>
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>,</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100">
-              <a:effectLst/>
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:effectLst/>
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>1991–2024</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" kern="1200">
-            <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </cdr:txBody>
-    </cdr:sp>
-  </cdr:relSizeAnchor>
-  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
-    <cdr:from>
-      <cdr:x>0.26343</cdr:x>
-      <cdr:y>0.42808</cdr:y>
-    </cdr:from>
-    <cdr:to>
-      <cdr:x>0.40511</cdr:x>
-      <cdr:y>0.59199</cdr:y>
-    </cdr:to>
-    <cdr:sp macro="" textlink="">
-      <cdr:nvSpPr>
-        <cdr:cNvPr id="5" name="TextBox 4">
-          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A9E084F5-0B96-630A-2881-BBE3FCD7E1A1}"/>
-            </a:ext>
-          </a:extLst>
-        </cdr:cNvPr>
-        <cdr:cNvSpPr txBox="1"/>
-      </cdr:nvSpPr>
-      <cdr:spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="1764462" y="1680456"/>
-          <a:ext cx="948970" cy="643440"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </cdr:spPr>
-      <cdr:txBody>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-            <a:t>DNA</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-            <a:t>sequencing,</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:effectLst/>
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>2001–22</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" kern="1200">
-            <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </cdr:txBody>
-    </cdr:sp>
-  </cdr:relSizeAnchor>
-  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
-    <cdr:from>
-      <cdr:x>0.13456</cdr:x>
-      <cdr:y>0.42957</cdr:y>
-    </cdr:from>
-    <cdr:to>
-      <cdr:x>0.19182</cdr:x>
-      <cdr:y>0.55779</cdr:y>
-    </cdr:to>
-    <cdr:sp macro="" textlink="">
-      <cdr:nvSpPr>
-        <cdr:cNvPr id="6" name="TextBox 5">
-          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1AE0DB7A-E029-B57F-9D5A-278C5057FA5B}"/>
-            </a:ext>
-          </a:extLst>
-        </cdr:cNvPr>
-        <cdr:cNvSpPr txBox="1"/>
-      </cdr:nvSpPr>
-      <cdr:spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="901258" y="1686307"/>
-          <a:ext cx="383526" cy="503337"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </cdr:spPr>
-      <cdr:txBody>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-            <a:t>AI</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:effectLst/>
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>,</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100">
-              <a:effectLst/>
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:effectLst/>
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>2021–26</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" kern="1200">
-            <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </cdr:txBody>
-    </cdr:sp>
-  </cdr:relSizeAnchor>
-  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
-    <cdr:from>
-      <cdr:x>0.8706</cdr:x>
-      <cdr:y>0.12194</cdr:y>
-    </cdr:from>
-    <cdr:to>
-      <cdr:x>0.99374</cdr:x>
-      <cdr:y>0.2462</cdr:y>
-    </cdr:to>
-    <cdr:sp macro="" textlink="">
-      <cdr:nvSpPr>
-        <cdr:cNvPr id="7" name="TextBox 6">
-          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{89558BC0-E47B-44E8-15AA-1CD6C980C277}"/>
-            </a:ext>
-          </a:extLst>
-        </cdr:cNvPr>
-        <cdr:cNvSpPr txBox="1"/>
-      </cdr:nvSpPr>
-      <cdr:spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="5831231" y="478680"/>
-          <a:ext cx="824839" cy="487791"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </cdr:spPr>
-      <cdr:txBody>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-            <a:t>Electricity,</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-            <a:t>1892–1973</a:t>
-          </a:r>
-        </a:p>
-      </cdr:txBody>
-    </cdr:sp>
-  </cdr:relSizeAnchor>
-  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
-    <cdr:from>
-      <cdr:x>0.00796</cdr:x>
-      <cdr:y>0</cdr:y>
-    </cdr:from>
-    <cdr:to>
-      <cdr:x>0.08745</cdr:x>
-      <cdr:y>0.099</cdr:y>
-    </cdr:to>
-    <cdr:sp macro="" textlink="">
-      <cdr:nvSpPr>
-        <cdr:cNvPr id="4" name="TextBox 3">
-          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9E6EFF4C-E325-4C3A-AC7D-7A0F249A747B}"/>
-            </a:ext>
-          </a:extLst>
-        </cdr:cNvPr>
-        <cdr:cNvSpPr txBox="1"/>
-      </cdr:nvSpPr>
-      <cdr:spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="53340" y="0"/>
-          <a:ext cx="532378" cy="388620"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </cdr:spPr>
-      <cdr:txBody>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:pPr algn="r"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-            <a:t>Starting</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-            <a:t>price</a:t>
-          </a:r>
-        </a:p>
-      </cdr:txBody>
-    </cdr:sp>
-  </cdr:relSizeAnchor>
-  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
-    <cdr:from>
-      <cdr:x>0.04601</cdr:x>
-      <cdr:y>0.1028</cdr:y>
-    </cdr:from>
-    <cdr:to>
-      <cdr:x>0.09846</cdr:x>
-      <cdr:y>0.17358</cdr:y>
-    </cdr:to>
-    <cdr:sp macro="" textlink="">
-      <cdr:nvSpPr>
-        <cdr:cNvPr id="8" name="TextBox 7">
-          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8660BA5-7038-65A7-9FF1-0F500B788276}"/>
-            </a:ext>
-          </a:extLst>
-        </cdr:cNvPr>
-        <cdr:cNvSpPr txBox="1"/>
-      </cdr:nvSpPr>
-      <cdr:spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="308164" y="403555"/>
-          <a:ext cx="351309" cy="277852"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </cdr:spPr>
-      <cdr:txBody>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:pPr algn="r"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-            <a:t>10x fall</a:t>
-          </a:r>
-        </a:p>
-      </cdr:txBody>
-    </cdr:sp>
-  </cdr:relSizeAnchor>
-  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
-    <cdr:from>
-      <cdr:x>0.02446</cdr:x>
-      <cdr:y>0.17746</cdr:y>
-    </cdr:from>
-    <cdr:to>
-      <cdr:x>0.09556</cdr:x>
-      <cdr:y>0.25212</cdr:y>
-    </cdr:to>
-    <cdr:sp macro="" textlink="">
-      <cdr:nvSpPr>
-        <cdr:cNvPr id="9" name="TextBox 8">
-          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6B7D3985-CC17-2DF7-E36A-C5B4D9537AAC}"/>
-            </a:ext>
-          </a:extLst>
-        </cdr:cNvPr>
-        <cdr:cNvSpPr txBox="1"/>
-      </cdr:nvSpPr>
-      <cdr:spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="163830" y="696634"/>
-          <a:ext cx="476227" cy="293083"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </cdr:spPr>
-      <cdr:txBody>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-            <a:t>100x</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
-        </a:p>
-      </cdr:txBody>
-    </cdr:sp>
-  </cdr:relSizeAnchor>
-  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
-    <cdr:from>
-      <cdr:x>0.0599</cdr:x>
-      <cdr:y>0.40353</cdr:y>
-    </cdr:from>
-    <cdr:to>
-      <cdr:x>0.0937</cdr:x>
-      <cdr:y>0.48983</cdr:y>
-    </cdr:to>
-    <cdr:sp macro="" textlink="">
-      <cdr:nvSpPr>
-        <cdr:cNvPr id="10" name="TextBox 9">
-          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9E65FA36-95D4-E093-4095-D9E3AA41C5E3}"/>
-            </a:ext>
-          </a:extLst>
-        </cdr:cNvPr>
-        <cdr:cNvSpPr txBox="1"/>
-      </cdr:nvSpPr>
-      <cdr:spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="401211" y="1584086"/>
-          <a:ext cx="226391" cy="338777"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </cdr:spPr>
-      <cdr:txBody>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
-        </a:p>
-      </cdr:txBody>
-    </cdr:sp>
-  </cdr:relSizeAnchor>
-  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
-    <cdr:from>
-      <cdr:x>0.06063</cdr:x>
-      <cdr:y>0.24666</cdr:y>
-    </cdr:from>
-    <cdr:to>
-      <cdr:x>0.09443</cdr:x>
-      <cdr:y>0.3056</cdr:y>
-    </cdr:to>
-    <cdr:sp macro="" textlink="">
-      <cdr:nvSpPr>
-        <cdr:cNvPr id="11" name="TextBox 1">
-          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0F0CBBC-B2A7-7545-154C-45F157FD73F0}"/>
-            </a:ext>
-          </a:extLst>
-        </cdr:cNvPr>
-        <cdr:cNvSpPr txBox="1"/>
-      </cdr:nvSpPr>
-      <cdr:spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="406077" y="968271"/>
-          <a:ext cx="226391" cy="231374"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </cdr:spPr>
-      <cdr:txBody>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="none" rtlCol="0"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:lvl1pPr marL="0" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl1pPr>
-          <a:lvl2pPr marL="457200" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl2pPr>
-          <a:lvl3pPr marL="914400" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl3pPr>
-          <a:lvl4pPr marL="1371600" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl4pPr>
-          <a:lvl5pPr marL="1828800" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl5pPr>
-          <a:lvl6pPr marL="2286000" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl6pPr>
-          <a:lvl7pPr marL="2743200" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl7pPr>
-          <a:lvl8pPr marL="3200400" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl8pPr>
-          <a:lvl9pPr marL="3657600" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl9pPr>
-        </a:lstStyle>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
-        </a:p>
-      </cdr:txBody>
-    </cdr:sp>
-  </cdr:relSizeAnchor>
-  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
-    <cdr:from>
-      <cdr:x>0.05951</cdr:x>
-      <cdr:y>0.32509</cdr:y>
-    </cdr:from>
-    <cdr:to>
-      <cdr:x>0.09331</cdr:x>
-      <cdr:y>0.38403</cdr:y>
-    </cdr:to>
-    <cdr:sp macro="" textlink="">
-      <cdr:nvSpPr>
-        <cdr:cNvPr id="13" name="TextBox 1">
-          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7DAA3E2A-F391-FAF9-BA1C-34832F8F390A}"/>
-            </a:ext>
-          </a:extLst>
-        </cdr:cNvPr>
-        <cdr:cNvSpPr txBox="1"/>
-      </cdr:nvSpPr>
-      <cdr:spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="398598" y="1276147"/>
-          <a:ext cx="226392" cy="231373"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </cdr:spPr>
-      <cdr:txBody>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="none" rtlCol="0"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:lvl1pPr marL="0" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl1pPr>
-          <a:lvl2pPr marL="457200" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl2pPr>
-          <a:lvl3pPr marL="914400" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl3pPr>
-          <a:lvl4pPr marL="1371600" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl4pPr>
-          <a:lvl5pPr marL="1828800" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl5pPr>
-          <a:lvl6pPr marL="2286000" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl6pPr>
-          <a:lvl7pPr marL="2743200" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl7pPr>
-          <a:lvl8pPr marL="3200400" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl8pPr>
-          <a:lvl9pPr marL="3657600" indent="0">
-            <a:defRPr sz="1100">
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl9pPr>
-        </a:lstStyle>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
-        </a:p>
-      </cdr:txBody>
-    </cdr:sp>
-  </cdr:relSizeAnchor>
-</c:userShapes>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -12194,15 +8852,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>354330</xdr:rowOff>
+      <xdr:colOff>325898</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>36304</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>487680</xdr:colOff>
+      <xdr:colOff>623078</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>73660</xdr:rowOff>
+      <xdr:rowOff>120890</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -12237,8 +8895,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>573075</xdr:colOff>
       <xdr:row>68</xdr:row>
       <xdr:rowOff>85090</xdr:rowOff>
     </xdr:to>
@@ -13033,7 +9691,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
     <cdr:from>
@@ -13112,11 +9770,11 @@
   </cdr:relSizeAnchor>
   <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
     <cdr:from>
-      <cdr:x>0.387</cdr:x>
+      <cdr:x>0.42123</cdr:x>
       <cdr:y>0.1999</cdr:y>
     </cdr:from>
     <cdr:to>
-      <cdr:x>0.52868</cdr:x>
+      <cdr:x>0.56291</cdr:x>
       <cdr:y>0.2709</cdr:y>
     </cdr:to>
     <cdr:sp macro="" textlink="">
@@ -13132,8 +9790,8 @@
       </cdr:nvSpPr>
       <cdr:spPr>
         <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="2592123" y="784726"/>
-          <a:ext cx="948970" cy="278716"/>
+          <a:off x="2819065" y="788022"/>
+          <a:ext cx="948198" cy="279887"/>
         </a:xfrm>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <a:avLst/>
@@ -13264,12 +9922,12 @@
   </cdr:relSizeAnchor>
   <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
     <cdr:from>
-      <cdr:x>0.26343</cdr:x>
-      <cdr:y>0.42808</cdr:y>
+      <cdr:x>0.30138</cdr:x>
+      <cdr:y>0.42981</cdr:y>
     </cdr:from>
     <cdr:to>
-      <cdr:x>0.40511</cdr:x>
-      <cdr:y>0.59199</cdr:y>
+      <cdr:x>0.44306</cdr:x>
+      <cdr:y>0.59372</cdr:y>
     </cdr:to>
     <cdr:sp macro="" textlink="">
       <cdr:nvSpPr>
@@ -13284,8 +9942,8 @@
       </cdr:nvSpPr>
       <cdr:spPr>
         <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="1764462" y="1680456"/>
-          <a:ext cx="948970" cy="643440"/>
+          <a:off x="2017015" y="1694329"/>
+          <a:ext cx="948199" cy="646146"/>
         </a:xfrm>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <a:avLst/>
@@ -13341,12 +9999,12 @@
   </cdr:relSizeAnchor>
   <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
     <cdr:from>
-      <cdr:x>0.13456</cdr:x>
-      <cdr:y>0.42957</cdr:y>
+      <cdr:x>0.18132</cdr:x>
+      <cdr:y>0.4313</cdr:y>
     </cdr:from>
     <cdr:to>
-      <cdr:x>0.19182</cdr:x>
-      <cdr:y>0.55779</cdr:y>
+      <cdr:x>0.23858</cdr:x>
+      <cdr:y>0.55952</cdr:y>
     </cdr:to>
     <cdr:sp macro="" textlink="">
       <cdr:nvSpPr>
@@ -13361,8 +10019,8 @@
       </cdr:nvSpPr>
       <cdr:spPr>
         <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="901258" y="1686307"/>
-          <a:ext cx="383526" cy="503337"/>
+          <a:off x="1213512" y="1700202"/>
+          <a:ext cx="383214" cy="505454"/>
         </a:xfrm>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <a:avLst/>
@@ -13474,12 +10132,12 @@
   </cdr:relSizeAnchor>
   <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
     <cdr:from>
-      <cdr:x>0.00796</cdr:x>
-      <cdr:y>0</cdr:y>
+      <cdr:x>0.01177</cdr:x>
+      <cdr:y>0.03968</cdr:y>
     </cdr:from>
     <cdr:to>
-      <cdr:x>0.08745</cdr:x>
-      <cdr:y>0.099</cdr:y>
+      <cdr:x>0.1507</cdr:x>
+      <cdr:y>0.09739</cdr:y>
     </cdr:to>
     <cdr:sp macro="" textlink="">
       <cdr:nvSpPr>
@@ -13494,8 +10152,8 @@
       </cdr:nvSpPr>
       <cdr:spPr>
         <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="53340" y="0"/>
-          <a:ext cx="532378" cy="388620"/>
+          <a:off x="78719" y="155521"/>
+          <a:ext cx="929351" cy="226238"/>
         </a:xfrm>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <a:avLst/>
@@ -13508,21 +10166,22 @@
           <a:pPr algn="r"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
             </a:rPr>
             <a:t>Starting</a:t>
           </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" kern="1200" baseline="0">
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
             </a:rPr>
-          </a:br>
+            <a:t> </a:t>
+          </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
             </a:rPr>
             <a:t>price</a:t>
           </a:r>
@@ -13532,12 +10191,12 @@
   </cdr:relSizeAnchor>
   <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
     <cdr:from>
-      <cdr:x>0.04601</cdr:x>
-      <cdr:y>0.1028</cdr:y>
+      <cdr:x>0.06013</cdr:x>
+      <cdr:y>0.10039</cdr:y>
     </cdr:from>
     <cdr:to>
-      <cdr:x>0.09846</cdr:x>
-      <cdr:y>0.17358</cdr:y>
+      <cdr:x>0.16559</cdr:x>
+      <cdr:y>0.17117</cdr:y>
     </cdr:to>
     <cdr:sp macro="" textlink="">
       <cdr:nvSpPr>
@@ -13552,8 +10211,8 @@
       </cdr:nvSpPr>
       <cdr:spPr>
         <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="308164" y="403555"/>
-          <a:ext cx="351309" cy="277852"/>
+          <a:off x="402231" y="393507"/>
+          <a:ext cx="705452" cy="277441"/>
         </a:xfrm>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <a:avLst/>
@@ -13566,10 +10225,10 @@
           <a:pPr algn="r"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
             </a:rPr>
-            <a:t>10x fall</a:t>
+            <a:t>10× cheaper</a:t>
           </a:r>
         </a:p>
       </cdr:txBody>
@@ -13577,11 +10236,11 @@
   </cdr:relSizeAnchor>
   <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
     <cdr:from>
-      <cdr:x>0.02446</cdr:x>
+      <cdr:x>0.03105</cdr:x>
       <cdr:y>0.17746</cdr:y>
     </cdr:from>
     <cdr:to>
-      <cdr:x>0.09556</cdr:x>
+      <cdr:x>0.13773</cdr:x>
       <cdr:y>0.25212</cdr:y>
     </cdr:to>
     <cdr:sp macro="" textlink="">
@@ -13597,8 +10256,8 @@
       </cdr:nvSpPr>
       <cdr:spPr>
         <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="163830" y="696634"/>
-          <a:ext cx="476227" cy="293083"/>
+          <a:off x="207697" y="695604"/>
+          <a:ext cx="713604" cy="292650"/>
         </a:xfrm>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <a:avLst/>
@@ -13611,112 +10270,43 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
             </a:rPr>
-            <a:t>100x</a:t>
+            <a:t>100</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:effectLst/>
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>×</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" kern="1200">
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+            </a:rPr>
+            <a:t> cheaper</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
             </a:rPr>
           </a:br>
           <a:br>
             <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
             </a:rPr>
           </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
-        </a:p>
-      </cdr:txBody>
-    </cdr:sp>
-  </cdr:relSizeAnchor>
-  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
-    <cdr:from>
-      <cdr:x>0.0599</cdr:x>
-      <cdr:y>0.40353</cdr:y>
-    </cdr:from>
-    <cdr:to>
-      <cdr:x>0.0937</cdr:x>
-      <cdr:y>0.48983</cdr:y>
-    </cdr:to>
-    <cdr:sp macro="" textlink="">
-      <cdr:nvSpPr>
-        <cdr:cNvPr id="10" name="TextBox 9">
-          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9E65FA36-95D4-E093-4095-D9E3AA41C5E3}"/>
-            </a:ext>
-          </a:extLst>
-        </cdr:cNvPr>
-        <cdr:cNvSpPr txBox="1"/>
-      </cdr:nvSpPr>
-      <cdr:spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="401211" y="1584086"/>
-          <a:ext cx="226391" cy="338777"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </cdr:spPr>
-      <cdr:txBody>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" kern="1200">
+            <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+            <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+          </a:endParaRPr>
         </a:p>
       </cdr:txBody>
     </cdr:sp>
@@ -13818,32 +10408,29 @@
           </a:lvl9pPr>
         </a:lstStyle>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" kern="1200">
+            <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+            <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+          </a:endParaRPr>
         </a:p>
       </cdr:txBody>
     </cdr:sp>
   </cdr:relSizeAnchor>
   <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
     <cdr:from>
-      <cdr:x>0.05951</cdr:x>
-      <cdr:y>0.32509</cdr:y>
+      <cdr:x>0.02352</cdr:x>
+      <cdr:y>0.25509</cdr:y>
     </cdr:from>
     <cdr:to>
-      <cdr:x>0.09331</cdr:x>
-      <cdr:y>0.38403</cdr:y>
+      <cdr:x>0.1302</cdr:x>
+      <cdr:y>0.32975</cdr:y>
     </cdr:to>
     <cdr:sp macro="" textlink="">
       <cdr:nvSpPr>
-        <cdr:cNvPr id="13" name="TextBox 1">
+        <cdr:cNvPr id="12" name="TextBox 1">
           <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7DAA3E2A-F391-FAF9-BA1C-34832F8F390A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C966B766-BB22-958D-04DF-C52D4AB984D1}"/>
             </a:ext>
           </a:extLst>
         </cdr:cNvPr>
@@ -13851,8 +10438,8 @@
       </cdr:nvSpPr>
       <cdr:spPr>
         <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="398598" y="1276147"/>
-          <a:ext cx="226392" cy="231373"/>
+          <a:off x="157389" y="1005568"/>
+          <a:ext cx="713963" cy="294315"/>
         </a:xfrm>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <a:avLst/>
@@ -13926,13 +10513,426 @@
           </a:lvl9pPr>
         </a:lstStyle>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100" kern="1200">
-              <a:latin typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="Cambria" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
             </a:rPr>
-            <a:t>.</a:t>
+            <a:t>1000</a:t>
           </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:effectLst/>
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>×</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" kern="1200">
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+            </a:rPr>
+            <a:t> cheaper</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" kern="1200">
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+            </a:rPr>
+          </a:br>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" kern="1200">
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+            </a:rPr>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" kern="1200">
+            <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+            <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.03193</cdr:x>
+      <cdr:y>0.48371</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.17751</cdr:x>
+      <cdr:y>0.55837</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="14" name="TextBox 1">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C966B766-BB22-958D-04DF-C52D4AB984D1}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="213609" y="1896016"/>
+          <a:ext cx="973780" cy="292650"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" kern="1200">
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+            </a:rPr>
+            <a:t>1 million</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:effectLst/>
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>×</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" kern="1200">
+            <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+            <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.0321</cdr:x>
+      <cdr:y>0.71648</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.17768</cdr:x>
+      <cdr:y>0.79114</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="15" name="TextBox 1">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{053B2150-99B6-1CF4-6E55-FBAA25B5F73B}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="214748" y="2808451"/>
+          <a:ext cx="973780" cy="292650"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" kern="1200">
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+            </a:rPr>
+            <a:t>1 billion</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:effectLst/>
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>×</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" kern="1200">
+            <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+            <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.00847</cdr:x>
+      <cdr:y>0.86882</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.17553</cdr:x>
+      <cdr:y>0.94348</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="16" name="TextBox 1">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{053B2150-99B6-1CF4-6E55-FBAA25B5F73B}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="56678" y="3405565"/>
+          <a:ext cx="1117490" cy="292650"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" kern="1200">
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+            </a:rPr>
+            <a:t>100</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" kern="1200" baseline="0">
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+            </a:rPr>
+            <a:t> b</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" kern="1200">
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+            </a:rPr>
+            <a:t>illion</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:effectLst/>
+              <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>×</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" kern="1200">
+            <a:latin typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+            <a:ea typeface="Inter" panose="02000503000000020004" pitchFamily="2" charset="0"/>
+          </a:endParaRPr>
         </a:p>
       </cdr:txBody>
     </cdr:sp>
@@ -13940,7 +10940,7 @@
 </c:userShapes>
 </file>
 
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
     <cdr:from>
@@ -14382,7 +11382,7 @@
 </c:userShapes>
 </file>
 
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -14887,7 +11887,7 @@
     <col min="5" max="5" width="14.26171875" customWidth="1"/>
     <col min="6" max="6" width="1.41796875" customWidth="1"/>
     <col min="7" max="7" width="14.26171875" customWidth="1"/>
-    <col min="8" max="8" width="6" customWidth="1"/>
+    <col min="8" max="8" width="6.89453125" customWidth="1"/>
     <col min="9" max="9" width="10.9453125" customWidth="1"/>
     <col min="22" max="29" width="10.89453125" customWidth="1"/>
   </cols>
@@ -14908,12 +11908,16 @@
       <c r="E1" s="50" t="s">
         <v>201</v>
       </c>
-      <c r="F1" s="51"/>
-      <c r="G1" s="58" t="s">
+      <c r="F1" s="50"/>
+      <c r="G1" s="68" t="s">
         <v>220</v>
       </c>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
+      <c r="H1" s="68" t="s">
+        <v>236</v>
+      </c>
+      <c r="I1" s="58" t="s">
+        <v>237</v>
+      </c>
       <c r="V1" s="11"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.55000000000000004">
@@ -15089,15 +12093,15 @@
         <v>0.47</v>
       </c>
       <c r="F7" s="52"/>
-      <c r="G7" s="57">
+      <c r="G7" s="65">
         <f t="shared" si="2"/>
         <v>0.6348782724359695</v>
       </c>
-      <c r="H7" s="59">
+      <c r="H7" s="66">
         <f>$G$7/G7</f>
         <v>1</v>
       </c>
-      <c r="I7" s="61">
+      <c r="I7" s="67">
         <f>(1-D7)^-4</f>
         <v>12.673498611808327</v>
       </c>
@@ -15266,11 +12270,11 @@
         <v>1</v>
       </c>
       <c r="M2">
-        <f>Table!$B11</f>
+        <f>Figure!$B11</f>
         <v>0</v>
       </c>
       <c r="N2">
-        <f>Table!$C11/100</f>
+        <f>Figure!$C11/100</f>
         <v>1</v>
       </c>
       <c r="O2">
@@ -15328,11 +12332,11 @@
         <v>1.3704928740696811</v>
       </c>
       <c r="M3">
-        <f>Table!$B12</f>
+        <f>Figure!$B12</f>
         <v>1.6163586584530094</v>
       </c>
       <c r="N3">
-        <f>Table!$C12/100</f>
+        <f>Figure!$C12/100</f>
         <v>1.6493911422653169E-2</v>
       </c>
       <c r="O3">
@@ -15390,11 +12394,11 @@
         <v>1.5817180939853757</v>
       </c>
       <c r="M4">
-        <f>Table!$B13</f>
+        <f>Figure!$B13</f>
         <v>4.7829586584530261</v>
       </c>
       <c r="N4">
-        <f>Table!$C13/100</f>
+        <f>Figure!$C13/100</f>
         <v>5.307518695827581E-6</v>
       </c>
       <c r="O4">

</xml_diff>